<commit_message>
Auto commit 21-07-2025 22:33:35.55
</commit_message>
<xml_diff>
--- a/Side Bar Files/GWD Data/3 Core Cable PRICE.xlsx
+++ b/Side Bar Files/GWD Data/3 Core Cable PRICE.xlsx
@@ -400,9 +400,15 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -826,7 +832,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA6F0FB-C978-426E-BF42-23C45514B9A6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8756D994-7D89-4635-8972-276E27A9B9A7}">
   <dimension ref="A1:G232"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>

</xml_diff>

<commit_message>
Auto commit 09-07-2026 16:57:44.38
</commit_message>
<xml_diff>
--- a/Side Bar Files/GWD Data/3 Core Cable PRICE.xlsx
+++ b/Side Bar Files/GWD Data/3 Core Cable PRICE.xlsx
@@ -367,25 +367,11 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment/>
       <protection/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -451,11 +437,11 @@
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="15" builtinId="5"/>
-    <cellStyle name="Currency" xfId="16" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
-    <cellStyle name="Comma" xfId="18" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="3" builtinId="7"/>
+    <cellStyle name="Comma" xfId="4" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="5" builtinId="6"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -832,7 +818,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8756D994-7D89-4635-8972-276E27A9B9A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D86AA3-DE4E-4FAD-95CD-7044C3A7BAA6}">
   <dimension ref="A1:G232"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>

</xml_diff>